<commit_message>
Adicionados as primeiras formulas
</commit_message>
<xml_diff>
--- a/Excel/CalcGrower_v0.1.xlsx
+++ b/Excel/CalcGrower_v0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jefferson\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A25E67F-7827-467A-86EF-AF14B37F6D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63897DF2-A9E3-422E-B6B0-4575DEA32A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{460B75DA-C666-464C-971D-95AEB43A337B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{460B75DA-C666-464C-971D-95AEB43A337B}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -33,8 +33,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -42,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="96">
   <si>
     <t>Fabricante</t>
   </si>
@@ -266,9 +264,6 @@
     <t>Molibdênio (Mo)</t>
   </si>
   <si>
-    <t>Totais</t>
-  </si>
-  <si>
     <t>N%</t>
   </si>
   <si>
@@ -305,13 +300,34 @@
     <t>Mo%</t>
   </si>
   <si>
-    <t>Coluna1</t>
-  </si>
-  <si>
     <t>Formula</t>
   </si>
   <si>
-    <t>-</t>
+    <t>Nutriente</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Macronutrientes</t>
+  </si>
+  <si>
+    <t>Micronutrientes</t>
+  </si>
+  <si>
+    <t>Elemnto Principal</t>
+  </si>
+  <si>
+    <t>Micro</t>
+  </si>
+  <si>
+    <t>ppm</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -492,7 +508,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -522,7 +538,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -552,284 +568,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="57">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
+  <dxfs count="59">
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1170,6 +924,50 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1225,6 +1023,16 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1232,7 +1040,7 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1246,6 +1054,7 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1253,22 +1062,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1276,22 +1086,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1299,22 +1110,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1322,22 +1134,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1345,22 +1158,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1368,22 +1182,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1391,22 +1206,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1414,22 +1230,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1437,22 +1254,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1460,22 +1278,23 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1483,7 +1302,295 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1555,16 +1662,37 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1577,62 +1705,6 @@
         </right>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
   </dxfs>
@@ -1698,8 +1770,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E7C143D1-2763-45E0-A650-B62B9F30D4B7}" name="tbFertilizantes" displayName="tbFertilizantes" ref="A1:T7" totalsRowShown="0" headerRowDxfId="55">
-  <autoFilter ref="A1:T7" xr:uid="{E7C143D1-2763-45E0-A650-B62B9F30D4B7}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E7C143D1-2763-45E0-A650-B62B9F30D4B7}" name="tbFertilizantes" displayName="tbFertilizantes" ref="A1:V7" totalsRowShown="0" headerRowDxfId="21">
+  <autoFilter ref="A1:V7" xr:uid="{E7C143D1-2763-45E0-A650-B62B9F30D4B7}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1720,35 +1792,39 @@
     <filterColumn colId="17" hiddenButton="1"/>
     <filterColumn colId="18" hiddenButton="1"/>
     <filterColumn colId="19" hiddenButton="1"/>
+    <filterColumn colId="20" hiddenButton="1"/>
+    <filterColumn colId="21" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{A2D5B959-4CFE-41FF-BC56-0ED245C25662}" name="ID" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{54153458-FF24-4BE8-B3E4-9333239EE6AA}" name="Produto" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{FAD8C287-0303-4CF4-ACB2-1DA5C6009CA4}" name="Fabricante" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{BC5F9AED-CB7E-4034-B0C1-52F67DFF7AC0}" name="Formula" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{AD0F1A8E-626E-4680-9E06-6F4AE92225D5}" name="N" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{C9064F87-9D4A-4F81-BA6E-3F989239C85C}" name="P" dataDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{B1E6223E-C0AE-462D-B234-3496FA6557FE}" name="K" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{87CA8122-2D4E-40D5-8337-3B1170425E83}" name="Ca" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{20D89E3E-02E5-45FB-951D-019143B8D0FD}" name="Mg" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{4331F3AA-3217-4802-8396-EB8F73E23B79}" name="S" dataDxfId="22"/>
-    <tableColumn id="11" xr3:uid="{8774BCE4-E672-4957-BEA8-4C83A072A375}" name="Fe" dataDxfId="21"/>
-    <tableColumn id="12" xr3:uid="{C439FC58-742E-466F-B739-BB7047BA2264}" name="Mn" dataDxfId="20"/>
-    <tableColumn id="13" xr3:uid="{CCF46CA3-6CA5-4697-9E1F-93ED13D77CD3}" name="Zn" dataDxfId="19"/>
-    <tableColumn id="14" xr3:uid="{7A1A50A1-E85A-4BAD-95F2-8203DA737C11}" name="B" dataDxfId="18"/>
-    <tableColumn id="15" xr3:uid="{713E21AF-495B-40E7-BBAB-95882468D61B}" name="Cu" dataDxfId="17"/>
-    <tableColumn id="16" xr3:uid="{95AB7424-53CC-469E-A672-316BEA2C5DD3}" name="Mo" dataDxfId="16"/>
-    <tableColumn id="17" xr3:uid="{F657BD02-0735-413F-999A-3AD63FD4BD12}" name="Solubilidade (g/L)" dataDxfId="15"/>
-    <tableColumn id="18" xr3:uid="{7D18331B-D187-40EA-A416-22BC6D802169}" name="Preço (R$/Kg)" dataDxfId="14"/>
-    <tableColumn id="19" xr3:uid="{517FA329-02F0-4B9D-8205-F5178B426D26}" name="Grupo de concentrado" dataDxfId="13"/>
-    <tableColumn id="20" xr3:uid="{09C2E469-2898-4054-BF94-7E1D2B019E71}" name="Observações" dataDxfId="12"/>
+  <tableColumns count="22">
+    <tableColumn id="1" xr3:uid="{A2D5B959-4CFE-41FF-BC56-0ED245C25662}" name="ID" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{54153458-FF24-4BE8-B3E4-9333239EE6AA}" name="Produto" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{FAD8C287-0303-4CF4-ACB2-1DA5C6009CA4}" name="Fabricante" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{BC5F9AED-CB7E-4034-B0C1-52F67DFF7AC0}" name="Formula" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{AD0F1A8E-626E-4680-9E06-6F4AE92225D5}" name="N" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{C9064F87-9D4A-4F81-BA6E-3F989239C85C}" name="P" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{B1E6223E-C0AE-462D-B234-3496FA6557FE}" name="K" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{87CA8122-2D4E-40D5-8337-3B1170425E83}" name="Ca" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{20D89E3E-02E5-45FB-951D-019143B8D0FD}" name="Mg" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{4331F3AA-3217-4802-8396-EB8F73E23B79}" name="S" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{8774BCE4-E672-4957-BEA8-4C83A072A375}" name="Fe" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{C439FC58-742E-466F-B739-BB7047BA2264}" name="Mn" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{CCF46CA3-6CA5-4697-9E1F-93ED13D77CD3}" name="Zn" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{7A1A50A1-E85A-4BAD-95F2-8203DA737C11}" name="B" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{713E21AF-495B-40E7-BBAB-95882468D61B}" name="Cu" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{95AB7424-53CC-469E-A672-316BEA2C5DD3}" name="Mo" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{F657BD02-0735-413F-999A-3AD63FD4BD12}" name="Solubilidade (g/L)" dataDxfId="4"/>
+    <tableColumn id="18" xr3:uid="{7D18331B-D187-40EA-A416-22BC6D802169}" name="Preço (R$/Kg)" dataDxfId="3"/>
+    <tableColumn id="19" xr3:uid="{517FA329-02F0-4B9D-8205-F5178B426D26}" name="Grupo de concentrado" dataDxfId="2"/>
+    <tableColumn id="20" xr3:uid="{09C2E469-2898-4054-BF94-7E1D2B019E71}" name="Observações" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{FF527B04-6A97-4781-B26B-5BE6D5F7E717}" name="Categoria" dataDxfId="0"/>
+    <tableColumn id="22" xr3:uid="{B9B62B91-2A31-4445-ADEA-C95319A4FBEE}" name="Elemnto Principal" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{36D45FC0-2870-4D2D-9F48-65A968840A8A}" name="tbCore" displayName="tbCore" ref="A1:AA7" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50" headerRowBorderDxfId="53" tableBorderDxfId="54" totalsRowBorderDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{36D45FC0-2870-4D2D-9F48-65A968840A8A}" name="tbCore" displayName="tbCore" ref="A1:AA7" totalsRowShown="0" headerRowDxfId="58" dataDxfId="56" headerRowBorderDxfId="57" tableBorderDxfId="55" totalsRowBorderDxfId="54">
   <autoFilter ref="A1:AA7" xr:uid="{36D45FC0-2870-4D2D-9F48-65A968840A8A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1779,71 +1855,95 @@
     <filterColumn colId="26" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="27">
-    <tableColumn id="1" xr3:uid="{76144110-7C5B-40DD-9FA1-1804EDDC887A}" name="Ferilizante" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{10BA7E9E-ECBA-43AF-8A4F-863888E51EB4}" name=" g/L" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{071368D0-EBC2-4032-93AC-5DB90A2BD224}" name="ID" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{071736F8-1715-4240-91AA-D56D2D50F809}" name="N%" dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{76144110-7C5B-40DD-9FA1-1804EDDC887A}" name="Ferilizante" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{10BA7E9E-ECBA-43AF-8A4F-863888E51EB4}" name=" g/L" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{071368D0-EBC2-4032-93AC-5DB90A2BD224}" name="ID" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{071736F8-1715-4240-91AA-D56D2D50F809}" name="N%" dataDxfId="50">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[N],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C20B8301-E9FA-4A62-B81D-CB29350E257D}" name="P%" dataDxfId="10">
+    <tableColumn id="5" xr3:uid="{C20B8301-E9FA-4A62-B81D-CB29350E257D}" name="P%" dataDxfId="49">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[P],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{D421A141-BF96-4F56-B9AC-B09E23DE53D5}" name="K%" dataDxfId="9">
+    <tableColumn id="6" xr3:uid="{D421A141-BF96-4F56-B9AC-B09E23DE53D5}" name="K%" dataDxfId="48">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[K],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{CDBD4152-9341-40E6-88A4-64B4D0CC74ED}" name="Ca%" dataDxfId="8">
+    <tableColumn id="7" xr3:uid="{CDBD4152-9341-40E6-88A4-64B4D0CC74ED}" name="Ca%" dataDxfId="47">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{45116017-A258-437E-8AC5-C287F946F1DD}" name="Mg%" dataDxfId="7">
+    <tableColumn id="8" xr3:uid="{45116017-A258-437E-8AC5-C287F946F1DD}" name="Mg%" dataDxfId="46">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5E6F012E-FB69-498B-B71E-2657778768C5}" name="S%" dataDxfId="6">
+    <tableColumn id="9" xr3:uid="{5E6F012E-FB69-498B-B71E-2657778768C5}" name="S%" dataDxfId="45">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[S],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{E297B97B-F266-4204-B736-ABABD73533F3}" name="Fe%" dataDxfId="5">
+    <tableColumn id="10" xr3:uid="{E297B97B-F266-4204-B736-ABABD73533F3}" name="Fe%" dataDxfId="44">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{62C497F4-2678-403F-A627-1FE9CF7127CE}" name="Mn%" dataDxfId="4">
+    <tableColumn id="11" xr3:uid="{62C497F4-2678-403F-A627-1FE9CF7127CE}" name="Mn%" dataDxfId="43">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{8B9DD9A9-951B-4A1F-AE92-E121ADA4F15D}" name="Zn%" dataDxfId="3">
+    <tableColumn id="12" xr3:uid="{8B9DD9A9-951B-4A1F-AE92-E121ADA4F15D}" name="Zn%" dataDxfId="42">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{33AF03BB-0283-4249-858B-C66710803B38}" name="B%" dataDxfId="2">
+    <tableColumn id="13" xr3:uid="{33AF03BB-0283-4249-858B-C66710803B38}" name="B%" dataDxfId="41">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[B],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{65D972A8-ED42-42E6-BF5D-48A1F25490F9}" name="Cu%" dataDxfId="1">
+    <tableColumn id="14" xr3:uid="{65D972A8-ED42-42E6-BF5D-48A1F25490F9}" name="Cu%" dataDxfId="40">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Cu],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{039C0F97-EF38-4A5C-86D3-A1DCA39C0276}" name="Mo%" dataDxfId="0">
+    <tableColumn id="15" xr3:uid="{039C0F97-EF38-4A5C-86D3-A1DCA39C0276}" name="Mo%" dataDxfId="39">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{577BC5FA-CDBC-48D9-834D-755B12F25F37}" name="N ppm" dataDxfId="44"/>
-    <tableColumn id="17" xr3:uid="{E1244B60-4B82-4279-A888-261864D52E49}" name="P ppm" dataDxfId="43"/>
-    <tableColumn id="18" xr3:uid="{C8DA11C8-87B1-411A-89D8-C3D52F849DB4}" name="K ppm" dataDxfId="42"/>
-    <tableColumn id="19" xr3:uid="{44B282B0-0A73-4207-9B02-E132BC73FB61}" name="Ca ppm" dataDxfId="41"/>
-    <tableColumn id="20" xr3:uid="{C952A124-2798-4536-A777-9F671ABA262F}" name="Mg ppm" dataDxfId="40"/>
-    <tableColumn id="21" xr3:uid="{C6CAD4D7-1D78-483B-9A41-4E1E64474A78}" name="S ppm" dataDxfId="39"/>
-    <tableColumn id="22" xr3:uid="{6C1FCF1D-7F4A-439A-8EFD-D97B424E9A71}" name="Fe ppm" dataDxfId="38"/>
-    <tableColumn id="23" xr3:uid="{B3DEFC6B-61B4-4702-9EF7-2775802B94C6}" name="Mn ppm" dataDxfId="37"/>
-    <tableColumn id="24" xr3:uid="{CFEB854B-DD96-4D8D-BC98-87FE925926E1}" name="Zn ppm" dataDxfId="36"/>
-    <tableColumn id="25" xr3:uid="{61AF59C0-E414-4BBB-913C-376B84FBBBBE}" name="B ppm" dataDxfId="35"/>
-    <tableColumn id="26" xr3:uid="{A344ECD4-6578-48B2-AF50-7AC37612C92E}" name="Cu ppm" dataDxfId="34"/>
-    <tableColumn id="27" xr3:uid="{464B7893-069D-4A89-A3FB-3FC3DF68B950}" name="Mo ppm" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{577BC5FA-CDBC-48D9-834D-755B12F25F37}" name="N ppm" dataDxfId="38">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="17" xr3:uid="{E1244B60-4B82-4279-A888-261864D52E49}" name="P ppm" dataDxfId="37">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="18" xr3:uid="{C8DA11C8-87B1-411A-89D8-C3D52F849DB4}" name="K ppm" dataDxfId="36">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="19" xr3:uid="{44B282B0-0A73-4207-9B02-E132BC73FB61}" name="Ca ppm" dataDxfId="35">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="20" xr3:uid="{C952A124-2798-4536-A777-9F671ABA262F}" name="Mg ppm" dataDxfId="34">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="21" xr3:uid="{C6CAD4D7-1D78-483B-9A41-4E1E64474A78}" name="S ppm" dataDxfId="33">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="22" xr3:uid="{6C1FCF1D-7F4A-439A-8EFD-D97B424E9A71}" name="Fe ppm" dataDxfId="32">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="23" xr3:uid="{B3DEFC6B-61B4-4702-9EF7-2775802B94C6}" name="Mn ppm" dataDxfId="31">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="24" xr3:uid="{CFEB854B-DD96-4D8D-BC98-87FE925926E1}" name="Zn ppm" dataDxfId="30">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="25" xr3:uid="{61AF59C0-E414-4BBB-913C-376B84FBBBBE}" name="B ppm" dataDxfId="29">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="26" xr3:uid="{A344ECD4-6578-48B2-AF50-7AC37612C92E}" name="Cu ppm" dataDxfId="28">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="27" xr3:uid="{464B7893-069D-4A89-A3FB-3FC3DF68B950}" name="Mo ppm" dataDxfId="27">
+      <calculatedColumnFormula>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{516A8680-E46F-45AF-98A3-60CA5DC72E09}" name="Tabela3" displayName="Tabela3" ref="A10:B22" totalsRowShown="0" headerRowDxfId="48" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{516A8680-E46F-45AF-98A3-60CA5DC72E09}" name="Tabela3" displayName="Tabela3" ref="A10:B22" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A10:B22" xr:uid="{516A8680-E46F-45AF-98A3-60CA5DC72E09}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{EBE2381E-6F61-4F4F-B83A-2D122EAF76D6}" name="Totais" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{ED3005D5-F393-4F6C-AAB1-DF3793BF166A}" name="Coluna1" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{EBE2381E-6F61-4F4F-B83A-2D122EAF76D6}" name="Nutriente" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{ED3005D5-F393-4F6C-AAB1-DF3793BF166A}" name="Total" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2155,7 +2255,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6620928F-272B-43F4-861A-5D8E0480B12C}">
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -2177,9 +2277,11 @@
     <col min="18" max="18" width="15.140625" customWidth="1"/>
     <col min="19" max="19" width="22.85546875" customWidth="1"/>
     <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="21" max="21" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>14</v>
       </c>
@@ -2190,7 +2292,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>41</v>
@@ -2240,8 +2342,14 @@
       <c r="T1" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -2253,45 +2361,33 @@
       <c r="E2" s="20">
         <v>14</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="F2" s="7"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7">
         <v>16</v>
       </c>
-      <c r="I2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
       <c r="S2" s="7" t="s">
         <v>26</v>
       </c>
       <c r="T2" s="7"/>
-    </row>
-    <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U2" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -2303,47 +2399,33 @@
       <c r="E3" s="7">
         <v>12</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="F3" s="7"/>
       <c r="G3" s="7">
         <v>45</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
       <c r="S3" s="7" t="s">
         <v>27</v>
       </c>
       <c r="T3" s="7"/>
-    </row>
-    <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U3" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2352,50 +2434,36 @@
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
-      <c r="E4" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="E4" s="7"/>
       <c r="F4" s="7">
         <v>51</v>
       </c>
       <c r="G4" s="7">
         <v>30</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="7" t="s">
         <v>27</v>
       </c>
       <c r="T4" s="7"/>
-    </row>
-    <row r="5" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V4" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -2404,50 +2472,36 @@
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
       <c r="I5" s="7">
         <v>9</v>
       </c>
       <c r="J5" s="7">
         <v>11</v>
       </c>
-      <c r="K5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
       <c r="S5" s="7" t="s">
         <v>27</v>
       </c>
       <c r="T5" s="7"/>
-    </row>
-    <row r="6" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U5" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -2456,50 +2510,36 @@
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
       <c r="G6" s="7">
         <v>50</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
       <c r="J6" s="7">
         <v>17</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
       <c r="S6" s="7" t="s">
         <v>27</v>
       </c>
       <c r="T6" s="7"/>
-    </row>
-    <row r="7" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U6" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V6" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
@@ -2511,21 +2551,11 @@
       <c r="E7" s="7">
         <v>4</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>89</v>
-      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
       <c r="K7" s="7">
         <v>7</v>
       </c>
@@ -2550,6 +2580,12 @@
         <v>27</v>
       </c>
       <c r="T7" s="7"/>
+      <c r="U7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="V7" s="8" t="s">
+        <v>93</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2651,6 +2687,7 @@
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.7109375" customWidth="1"/>
     <col min="20" max="20" width="10.42578125" customWidth="1"/>
     <col min="22" max="22" width="9.7109375" customWidth="1"/>
@@ -2671,40 +2708,40 @@
         <v>14</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>86</v>
       </c>
       <c r="P1" s="5" t="s">
         <v>50</v>
@@ -2753,9 +2790,9 @@
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[N],0)</f>
         <v>14</v>
       </c>
-      <c r="E2" s="14" t="str">
+      <c r="E2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[P],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="F2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[K],0)</f>
@@ -2765,50 +2802,86 @@
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</f>
         <v>16</v>
       </c>
-      <c r="H2" s="14" t="str">
+      <c r="H2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</f>
-        <v>-</v>
-      </c>
-      <c r="I2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="I2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[S],0)</f>
-        <v>-</v>
-      </c>
-      <c r="J2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="J2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</f>
-        <v>-</v>
-      </c>
-      <c r="K2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="L2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="M2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="M2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[B],0)</f>
-        <v>-</v>
-      </c>
-      <c r="N2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="N2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Cu],0)</f>
-        <v>-</v>
-      </c>
-      <c r="O2" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="O2" s="14">
         <f>_xlfn.XLOOKUP(A2,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</f>
-        <v>-</v>
-      </c>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="14"/>
-      <c r="V2" s="14"/>
-      <c r="W2" s="14"/>
-      <c r="X2" s="14"/>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="15"/>
+        <v>0</v>
+      </c>
+      <c r="P2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="S2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="T2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="U2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="V2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="W2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="X2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Y2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="AA2" s="15">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
@@ -2820,62 +2893,98 @@
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[N],0)</f>
         <v>12</v>
       </c>
-      <c r="E3" s="14" t="str">
+      <c r="E3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[P],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="F3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[K],0)</f>
         <v>45</v>
       </c>
-      <c r="G3" s="14" t="str">
+      <c r="G3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</f>
-        <v>-</v>
-      </c>
-      <c r="H3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="H3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</f>
-        <v>-</v>
-      </c>
-      <c r="I3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="I3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[S],0)</f>
-        <v>-</v>
-      </c>
-      <c r="J3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="J3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</f>
-        <v>-</v>
-      </c>
-      <c r="K3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="L3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="M3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="M3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[B],0)</f>
-        <v>-</v>
-      </c>
-      <c r="N3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="N3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Cu],0)</f>
-        <v>-</v>
-      </c>
-      <c r="O3" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="O3" s="14">
         <f>_xlfn.XLOOKUP(A3,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</f>
-        <v>-</v>
-      </c>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-      <c r="W3" s="14"/>
-      <c r="X3" s="14"/>
-      <c r="Y3" s="14"/>
-      <c r="Z3" s="14"/>
-      <c r="AA3" s="15"/>
+        <v>0</v>
+      </c>
+      <c r="P3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="R3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="S3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="T3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="U3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="V3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="W3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="X3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Y3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Z3" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="AA3" s="15">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -2883,9 +2992,9 @@
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="7"/>
-      <c r="D4" s="14" t="str">
+      <c r="D4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[N],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="E4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[P],0)</f>
@@ -2895,54 +3004,90 @@
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[K],0)</f>
         <v>30</v>
       </c>
-      <c r="G4" s="14" t="str">
+      <c r="G4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</f>
-        <v>-</v>
-      </c>
-      <c r="H4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="H4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</f>
-        <v>-</v>
-      </c>
-      <c r="I4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="I4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[S],0)</f>
-        <v>-</v>
-      </c>
-      <c r="J4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</f>
-        <v>-</v>
-      </c>
-      <c r="K4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="L4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="M4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="M4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[B],0)</f>
-        <v>-</v>
-      </c>
-      <c r="N4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="N4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Cu],0)</f>
-        <v>-</v>
-      </c>
-      <c r="O4" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="O4" s="14">
         <f>_xlfn.XLOOKUP(A4,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</f>
-        <v>-</v>
-      </c>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="15"/>
+        <v>0</v>
+      </c>
+      <c r="P4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Q4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="R4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="S4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="T4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="U4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="V4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="W4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="X4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="AA4" s="15">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -2950,21 +3095,21 @@
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="7"/>
-      <c r="D5" s="14" t="str">
+      <c r="D5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[N],0)</f>
-        <v>-</v>
-      </c>
-      <c r="E5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="E5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[P],0)</f>
-        <v>-</v>
-      </c>
-      <c r="F5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="F5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[K],0)</f>
-        <v>-</v>
-      </c>
-      <c r="G5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="G5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="H5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</f>
@@ -2974,42 +3119,78 @@
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[S],0)</f>
         <v>11</v>
       </c>
-      <c r="J5" s="14" t="str">
+      <c r="J5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</f>
-        <v>-</v>
-      </c>
-      <c r="K5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="L5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="M5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="M5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[B],0)</f>
-        <v>-</v>
-      </c>
-      <c r="N5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="N5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Cu],0)</f>
-        <v>-</v>
-      </c>
-      <c r="O5" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="O5" s="14">
         <f>_xlfn.XLOOKUP(A5,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</f>
-        <v>-</v>
-      </c>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="14"/>
-      <c r="U5" s="14"/>
-      <c r="V5" s="14"/>
-      <c r="W5" s="14"/>
-      <c r="X5" s="14"/>
-      <c r="Y5" s="14"/>
-      <c r="Z5" s="14"/>
-      <c r="AA5" s="15"/>
+        <v>0</v>
+      </c>
+      <c r="P5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="S5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="U5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="V5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="W5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="X5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="15">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
@@ -3017,66 +3198,102 @@
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="7"/>
-      <c r="D6" s="14" t="str">
+      <c r="D6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[N],0)</f>
-        <v>-</v>
-      </c>
-      <c r="E6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="E6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[P],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="F6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[K],0)</f>
         <v>50</v>
       </c>
-      <c r="G6" s="14" t="str">
+      <c r="G6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</f>
-        <v>-</v>
-      </c>
-      <c r="H6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="H6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[S],0)</f>
         <v>17</v>
       </c>
-      <c r="J6" s="14" t="str">
+      <c r="J6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</f>
-        <v>-</v>
-      </c>
-      <c r="K6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="L6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="L6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Zn],0)</f>
-        <v>-</v>
-      </c>
-      <c r="M6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="M6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[B],0)</f>
-        <v>-</v>
-      </c>
-      <c r="N6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="N6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Cu],0)</f>
-        <v>-</v>
-      </c>
-      <c r="O6" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="O6" s="14">
         <f>_xlfn.XLOOKUP(A6,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</f>
-        <v>-</v>
-      </c>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="14"/>
-      <c r="S6" s="14"/>
-      <c r="T6" s="14"/>
-      <c r="U6" s="14"/>
-      <c r="V6" s="14"/>
-      <c r="W6" s="14"/>
-      <c r="X6" s="14"/>
-      <c r="Y6" s="14"/>
-      <c r="Z6" s="14"/>
-      <c r="AA6" s="15"/>
+        <v>0</v>
+      </c>
+      <c r="P6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="S6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="V6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="W6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="X6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="14">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="15">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
@@ -3088,25 +3305,25 @@
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[N],0)</f>
         <v>4</v>
       </c>
-      <c r="E7" s="16" t="str">
+      <c r="E7" s="16">
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[P],0)</f>
-        <v>-</v>
-      </c>
-      <c r="F7" s="16" t="str">
+        <v>0</v>
+      </c>
+      <c r="F7" s="16">
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[K],0)</f>
-        <v>-</v>
-      </c>
-      <c r="G7" s="16" t="str">
+        <v>0</v>
+      </c>
+      <c r="G7" s="16">
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[Ca],0)</f>
-        <v>-</v>
-      </c>
-      <c r="H7" s="16" t="str">
+        <v>0</v>
+      </c>
+      <c r="H7" s="16">
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[Mg],0)</f>
-        <v>-</v>
-      </c>
-      <c r="I7" s="16" t="str">
+        <v>0</v>
+      </c>
+      <c r="I7" s="16">
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[S],0)</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="J7" s="16">
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[Fe],0)</f>
@@ -3132,98 +3349,170 @@
         <f>_xlfn.XLOOKUP(A7,tbFertilizantes[Produto],tbFertilizantes[Mo],0)</f>
         <v>0.1</v>
       </c>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="16"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="16"/>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-      <c r="AA7" s="17"/>
+      <c r="P7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[N%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[P%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="R7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[K%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="S7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Ca%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="T7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mg%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="U7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[S%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="V7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Fe%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="W7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="X7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Zn%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[B%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="16">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Cu%]]*10</f>
+        <v>0</v>
+      </c>
+      <c r="AA7" s="17">
+        <f>tbCore[[#This Row],[ g/L]]*tbCore[[#This Row],[Mo%]]*10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="19"/>
+      <c r="B11" s="19">
+        <f>SUM(tbCore[N ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="19"/>
+      <c r="B12" s="19">
+        <f>SUM(tbCore[P ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="19"/>
+      <c r="B13" s="19">
+        <f>SUM(tbCore[K ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="19"/>
+      <c r="B14" s="19">
+        <f>SUM(tbCore[Ca ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="19"/>
+      <c r="B15" s="19">
+        <f>SUM(tbCore[Mg ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="19"/>
+      <c r="B16" s="19">
+        <f>SUM(tbCore[S ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="19"/>
+      <c r="B17" s="19">
+        <f>SUM(tbCore[Fe ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="19"/>
+      <c r="B18" s="19">
+        <f>SUM(tbCore[Mn ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="19"/>
+      <c r="B19" s="19">
+        <f>SUM(tbCore[Zn ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="19"/>
+      <c r="B20" s="19">
+        <f>SUM(tbCore[B ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="19"/>
+      <c r="B21" s="19">
+        <f>SUM(tbCore[Cu ppm])</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="19">
+        <f>SUM(tbCore[Mo ppm])</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -3231,14 +3520,127 @@
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
   </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6E3A5C77-7B09-4B7F-86F4-56AC8A4C38A6}">
+          <x14:formula1>
+            <xm:f>Fertilizante!$B$2:$B$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>A2:A7</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20218DE9-EE45-4D44-885E-A900808ADB4D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="21"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="22"/>
+      <c r="C3" s="21"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="21"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="21"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="22"/>
+      <c r="C6" s="21"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="21"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="21"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="21"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="C10" s="21"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="22"/>
+      <c r="C11" s="21"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="22"/>
+      <c r="C12" s="21"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="22"/>
+      <c r="C13" s="21"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>